<commit_message>
new 12mo version with customer acquisition date
</commit_message>
<xml_diff>
--- a/picha12mo/data_dict_en.xlsx
+++ b/picha12mo/data_dict_en.xlsx
@@ -15,17 +15,17 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">Codes!$A$1:$D$14</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Columns!$A$1:$K$100</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Columns!$A$1:$K$103</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">Notes!$A$1:$B$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Overview!$A$3:$D$10</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Relationships!$A$1:$E$7</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">Relationships!$A$1:$E$8</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="718" uniqueCount="391">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="739" uniqueCount="399">
   <si>
     <t>Table</t>
   </si>
@@ -105,7 +105,7 @@
     <t>PiCha Tea House — Data Dictionary (picha12mo.duckdb)</t>
   </si>
   <si>
-    <t>2026-01-01 to 2026-12-31 · 7 tables · 99 columns</t>
+    <t>2026-01-01 to 2026-12-31 · 7 tables · 102 columns</t>
   </si>
   <si>
     <t>Column</t>
@@ -252,9 +252,15 @@
     <t>age_group</t>
   </si>
   <si>
+    <t>dob</t>
+  </si>
+  <si>
     <t>gender</t>
   </si>
   <si>
+    <t>mobile</t>
+  </si>
+  <si>
     <t>income_segment</t>
   </si>
   <si>
@@ -273,6 +279,9 @@
     <t>acquisition_date</t>
   </si>
   <si>
+    <t>home_store_id</t>
+  </si>
+  <si>
     <t>sku_name</t>
   </si>
   <si>
@@ -570,9 +579,15 @@
     <t>Age cohort.</t>
   </si>
   <si>
+    <t>Date of birth. The customer's age on 2026-01-01 falls inside their age_group (Older_36plus: 36–60).</t>
+  </si>
+  <si>
     <t>Self-reported gender.</t>
   </si>
   <si>
+    <t>Mobile phone number (unique per customer), Thai format 0XX-XXX-XXXX starting 06/08/09. Synthetic.</t>
+  </si>
+  <si>
     <t>Income tier, assigned from the age-group distribution.</t>
   </si>
   <si>
@@ -588,7 +603,10 @@
     <t>Default sweetness pattern; 'adaptive' = no fixed pattern.</t>
   </si>
   <si>
-    <t>Date the customer joined. No order references a customer before this date.</t>
+    <t>Date the customer joined = date of their first purchase. Dates before 2026 are customers who joined in 2025 (pre-existing base); a few sign-ups never buy. No order references a customer before this date.</t>
+  </si>
+  <si>
+    <t>Store where the customer joined and places most (~85%) of their orders; the rest go to a backup store.</t>
   </si>
   <si>
     <t>Unique product identifier. 1–20 = core menu; 21–30 = new items launched during 2026.</t>
@@ -744,7 +762,7 @@
     <t>0</t>
   </si>
   <si>
-    <t>1001</t>
+    <t>1000</t>
   </si>
   <si>
     <t>85.00</t>
@@ -765,7 +783,7 @@
     <t>4.80</t>
   </si>
   <si>
-    <t>39.44</t>
+    <t>37.48</t>
   </si>
   <si>
     <t>3.00</t>
@@ -774,7 +792,10 @@
     <t>85</t>
   </si>
   <si>
-    <t>1000</t>
+    <t>1965-01-11</t>
+  </si>
+  <si>
+    <t>2025-03-01</t>
   </si>
   <si>
     <t>500</t>
@@ -795,9 +816,6 @@
     <t>0.65</t>
   </si>
   <si>
-    <t>2025-03-01</t>
-  </si>
-  <si>
     <t>20</t>
   </si>
   <si>
@@ -849,7 +867,7 @@
     <t>654.00</t>
   </si>
   <si>
-    <t>123.40</t>
+    <t>122.60</t>
   </si>
   <si>
     <t>30.00</t>
@@ -861,7 +879,7 @@
     <t>56.00</t>
   </si>
   <si>
-    <t>704.00</t>
+    <t>687.00</t>
   </si>
   <si>
     <t>248.08</t>
@@ -876,7 +894,7 @@
     <t>7.20</t>
   </si>
   <si>
-    <t>333.08</t>
+    <t>309.94</t>
   </si>
   <si>
     <t>14.70</t>
@@ -897,7 +915,7 @@
     <t>183</t>
   </si>
   <si>
-    <t>36.60</t>
+    <t>36.40</t>
   </si>
   <si>
     <t>183.00</t>
@@ -906,7 +924,7 @@
     <t>73.20</t>
   </si>
   <si>
-    <t>2026-12-30</t>
+    <t>2008-01-01</t>
   </si>
   <si>
     <t>700</t>
@@ -957,7 +975,7 @@
     <t>direct, YumDash, C2U</t>
   </si>
   <si>
-    <t>ICONSIAMEVE, FLAVOR50, BUILDER3, MALLCOMBO, WELCOME20, MORNING15, HAPPY2FOR1</t>
+    <t>BUILDER3, ICONSIAMEVE, FLAVOR50, MORNING15, HAPPY2FOR1, WELCOME20, MALLCOMBO</t>
   </si>
   <si>
     <t>sunny, cloudy, rainy</t>
@@ -978,6 +996,9 @@
     <t>male, female</t>
   </si>
   <si>
+    <t>e.g. 063-253-1125, 062-838-1255, 092-271-9391</t>
+  </si>
+  <si>
     <t>mid, high, low</t>
   </si>
   <si>
@@ -990,10 +1011,10 @@
     <t>full, less_sweet, adaptive</t>
   </si>
   <si>
-    <t>e.g. Glutinous Green Milk Tea L, Pu'er Milk Tea R, Osmanthus Milk Tea L</t>
-  </si>
-  <si>
-    <t>milk_tea, fruit_tea, blended, pure_tea, cold_brew</t>
+    <t>e.g. Tie Guan Yin Milk Tea R, Jasmine Milk Tea R, Peach Jasmine Tea L</t>
+  </si>
+  <si>
+    <t>milk_tea, fruit_tea, pure_tea, blended, cold_brew</t>
   </si>
   <si>
     <t>e.g. jasmine, glutinous_green, tie_guan_yin</t>
@@ -1005,16 +1026,16 @@
     <t>medium, low, high</t>
   </si>
   <si>
-    <t>PiCha Siam Square, PiCha Park Silom, PiCha ICONSIAM, PiCha Vanit Village, PiCha centralwOrld, PiCha Exchange Tower</t>
-  </si>
-  <si>
-    <t>office, mixed_use, mall, mall_flagship, street</t>
-  </si>
-  <si>
-    <t>Pathum Wan, Khlong Toei, Khlong San, Bang Rak, Ratchathewi</t>
-  </si>
-  <si>
-    <t>power outage, equipment failure, water supply cut, street flooding, building maintenance</t>
+    <t>PiCha Siam Square, PiCha Park Silom, PiCha Vanit Village, PiCha centralwOrld, PiCha Exchange Tower, PiCha ICONSIAM</t>
+  </si>
+  <si>
+    <t>office, mixed_use, mall_flagship, mall, street</t>
+  </si>
+  <si>
+    <t>Pathum Wan, Bang Rak, Ratchathewi, Khlong Toei, Khlong San</t>
+  </si>
+  <si>
+    <t>power outage, water supply cut, equipment failure, street flooding, building maintenance</t>
   </si>
   <si>
     <t>From (child)</t>
@@ -1038,6 +1059,9 @@
     <t>transactions.customer_id</t>
   </si>
   <si>
+    <t>customers.home_store_id</t>
+  </si>
+  <si>
     <t>order_items.transaction_id</t>
   </si>
   <si>
@@ -1182,7 +1206,7 @@
     <t>order_items.net_line_sales_thb = unit_list_price_thb − line_discount_thb</t>
   </si>
   <si>
-    <t>69% of orders have NULL customer_id (anonymous).</t>
+    <t>71% of orders have NULL customer_id (anonymous). About a quarter of customers joined in 2025; new customers join with their first purchase, mostly at busy times, at newly opened stores and after menu drops. Customers buy at their home store and churn after a few months.</t>
   </si>
   <si>
     <t>Core SKUs 1–20 cost 5 THB more from 2026-07-01 (see price_history). Delivery orders carry a 6–18% markup on unit_list_price_thb.</t>
@@ -1712,7 +1736,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:K100"/>
+  <dimension ref="A1:K103"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="15.7109375" style="1" customWidth="1"/>
@@ -1770,13 +1794,13 @@
         <v>11</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>135</v>
+        <v>138</v>
       </c>
       <c r="F2" s="1">
         <v>0</v>
@@ -1788,10 +1812,10 @@
         <v>385595</v>
       </c>
       <c r="I2" s="1" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="J2" s="1" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
     </row>
     <row r="3" spans="1:11">
@@ -1802,10 +1826,10 @@
         <v>36</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>136</v>
+        <v>139</v>
       </c>
       <c r="F3" s="1">
         <v>0</v>
@@ -1817,10 +1841,10 @@
         <v>380766</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="J3" s="1" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="4" spans="1:11">
@@ -1831,10 +1855,10 @@
         <v>37</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="F4" s="1">
         <v>0</v>
@@ -1846,10 +1870,10 @@
         <v>365</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>236</v>
+        <v>242</v>
       </c>
       <c r="J4" s="1" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
     </row>
     <row r="5" spans="1:11">
@@ -1860,10 +1884,10 @@
         <v>38</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>138</v>
+        <v>141</v>
       </c>
       <c r="F5" s="1">
         <v>0</v>
@@ -1875,10 +1899,10 @@
         <v>14</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>237</v>
+        <v>243</v>
       </c>
       <c r="J5" s="1" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
     </row>
     <row r="6" spans="1:11">
@@ -1889,10 +1913,10 @@
         <v>39</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>139</v>
+        <v>142</v>
       </c>
       <c r="F6" s="1">
         <v>0</v>
@@ -1904,7 +1928,7 @@
         <v>7</v>
       </c>
       <c r="K6" s="1" t="s">
-        <v>307</v>
+        <v>313</v>
       </c>
     </row>
     <row r="7" spans="1:11">
@@ -1915,10 +1939,10 @@
         <v>40</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>140</v>
+        <v>143</v>
       </c>
       <c r="F7" s="1">
         <v>0</v>
@@ -1930,10 +1954,10 @@
         <v>7</v>
       </c>
       <c r="I7" s="1" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="J7" s="1" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
     </row>
     <row r="8" spans="1:11">
@@ -1944,10 +1968,10 @@
         <v>41</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>141</v>
+        <v>144</v>
       </c>
       <c r="F8" s="1">
         <v>0</v>
@@ -1959,10 +1983,10 @@
         <v>12</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="J8" s="1" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9" spans="1:11">
@@ -1973,13 +1997,13 @@
         <v>15</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>129</v>
+        <v>132</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>142</v>
+        <v>145</v>
       </c>
       <c r="F9" s="1">
         <v>0</v>
@@ -1991,10 +2015,10 @@
         <v>6</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="J9" s="1" t="s">
-        <v>252</v>
+        <v>259</v>
       </c>
     </row>
     <row r="10" spans="1:11">
@@ -2005,10 +2029,10 @@
         <v>42</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E10" s="1" t="s">
-        <v>143</v>
+        <v>146</v>
       </c>
       <c r="F10" s="1">
         <v>0</v>
@@ -2020,7 +2044,7 @@
         <v>3</v>
       </c>
       <c r="K10" s="1" t="s">
-        <v>308</v>
+        <v>314</v>
       </c>
     </row>
     <row r="11" spans="1:11">
@@ -2031,10 +2055,10 @@
         <v>43</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E11" s="1" t="s">
-        <v>144</v>
+        <v>147</v>
       </c>
       <c r="F11" s="1">
         <v>0</v>
@@ -2046,7 +2070,7 @@
         <v>3</v>
       </c>
       <c r="K11" s="1" t="s">
-        <v>309</v>
+        <v>315</v>
       </c>
     </row>
     <row r="12" spans="1:11">
@@ -2057,28 +2081,28 @@
         <v>13</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>145</v>
+        <v>148</v>
       </c>
       <c r="F12" s="1">
-        <v>264257</v>
+        <v>273430</v>
       </c>
       <c r="G12" s="1">
-        <v>68.5</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="H12" s="1">
-        <v>5366</v>
+        <v>5819</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>239</v>
+        <v>245</v>
       </c>
       <c r="J12" s="1" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
     </row>
     <row r="13" spans="1:11">
@@ -2089,10 +2113,10 @@
         <v>44</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E13" s="1" t="s">
-        <v>146</v>
+        <v>149</v>
       </c>
       <c r="F13" s="1">
         <v>0</v>
@@ -2104,10 +2128,10 @@
         <v>4</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="J13" s="1" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
     </row>
     <row r="14" spans="1:11">
@@ -2118,10 +2142,10 @@
         <v>45</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E14" s="1" t="s">
-        <v>147</v>
+        <v>150</v>
       </c>
       <c r="F14" s="1">
         <v>0</v>
@@ -2133,10 +2157,10 @@
         <v>555</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>240</v>
+        <v>246</v>
       </c>
       <c r="J14" s="1" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
     </row>
     <row r="15" spans="1:11">
@@ -2147,10 +2171,10 @@
         <v>46</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>148</v>
+        <v>151</v>
       </c>
       <c r="F15" s="1">
         <v>0</v>
@@ -2159,13 +2183,13 @@
         <v>0</v>
       </c>
       <c r="H15" s="1">
-        <v>5691</v>
+        <v>6019</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="J15" s="1" t="s">
-        <v>274</v>
+        <v>280</v>
       </c>
     </row>
     <row r="16" spans="1:11">
@@ -2176,10 +2200,10 @@
         <v>47</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E16" s="1" t="s">
-        <v>149</v>
+        <v>152</v>
       </c>
       <c r="F16" s="1">
         <v>0</v>
@@ -2191,10 +2215,10 @@
         <v>2</v>
       </c>
       <c r="I16" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="J16" s="1" t="s">
-        <v>275</v>
+        <v>281</v>
       </c>
     </row>
     <row r="17" spans="1:11">
@@ -2205,10 +2229,10 @@
         <v>48</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E17" s="1" t="s">
-        <v>150</v>
+        <v>153</v>
       </c>
       <c r="F17" s="1">
         <v>0</v>
@@ -2220,10 +2244,10 @@
         <v>62</v>
       </c>
       <c r="I17" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="J17" s="1" t="s">
-        <v>276</v>
+        <v>282</v>
       </c>
     </row>
     <row r="18" spans="1:11">
@@ -2234,10 +2258,10 @@
         <v>49</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="F18" s="1">
         <v>0</v>
@@ -2249,10 +2273,10 @@
         <v>55</v>
       </c>
       <c r="I18" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="J18" s="1" t="s">
-        <v>277</v>
+        <v>283</v>
       </c>
     </row>
     <row r="19" spans="1:11">
@@ -2263,10 +2287,10 @@
         <v>50</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E19" s="1" t="s">
-        <v>152</v>
+        <v>155</v>
       </c>
       <c r="F19" s="1">
         <v>0</v>
@@ -2275,13 +2299,13 @@
         <v>0</v>
       </c>
       <c r="H19" s="1">
-        <v>33199</v>
+        <v>28741</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="J19" s="1" t="s">
-        <v>278</v>
+        <v>284</v>
       </c>
     </row>
     <row r="20" spans="1:11">
@@ -2292,10 +2316,10 @@
         <v>51</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E20" s="1" t="s">
-        <v>153</v>
+        <v>156</v>
       </c>
       <c r="F20" s="1">
         <v>0</v>
@@ -2304,13 +2328,13 @@
         <v>0</v>
       </c>
       <c r="H20" s="1">
-        <v>19899</v>
+        <v>19927</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="J20" s="1" t="s">
-        <v>279</v>
+        <v>285</v>
       </c>
     </row>
     <row r="21" spans="1:11">
@@ -2321,10 +2345,10 @@
         <v>52</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E21" s="1" t="s">
-        <v>154</v>
+        <v>157</v>
       </c>
       <c r="F21" s="1">
         <v>0</v>
@@ -2336,10 +2360,10 @@
         <v>7</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>244</v>
+        <v>250</v>
       </c>
       <c r="J21" s="1" t="s">
-        <v>280</v>
+        <v>286</v>
       </c>
     </row>
     <row r="22" spans="1:11">
@@ -2350,10 +2374,10 @@
         <v>53</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E22" s="1" t="s">
-        <v>155</v>
+        <v>158</v>
       </c>
       <c r="F22" s="1">
         <v>0</v>
@@ -2362,13 +2386,13 @@
         <v>0</v>
       </c>
       <c r="H22" s="1">
-        <v>10080</v>
+        <v>10141</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="J22" s="1" t="s">
-        <v>281</v>
+        <v>287</v>
       </c>
     </row>
     <row r="23" spans="1:11">
@@ -2379,10 +2403,10 @@
         <v>54</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E23" s="1" t="s">
-        <v>156</v>
+        <v>159</v>
       </c>
       <c r="F23" s="1">
         <v>0</v>
@@ -2394,10 +2418,10 @@
         <v>4</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>245</v>
+        <v>251</v>
       </c>
       <c r="J23" s="1" t="s">
-        <v>282</v>
+        <v>288</v>
       </c>
     </row>
     <row r="24" spans="1:11">
@@ -2408,10 +2432,10 @@
         <v>55</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E24" s="1" t="s">
-        <v>157</v>
+        <v>160</v>
       </c>
       <c r="F24" s="1">
         <v>0</v>
@@ -2420,13 +2444,13 @@
         <v>0</v>
       </c>
       <c r="H24" s="1">
-        <v>22250</v>
+        <v>21140</v>
       </c>
       <c r="I24" s="1" t="s">
-        <v>246</v>
+        <v>252</v>
       </c>
       <c r="J24" s="1" t="s">
-        <v>283</v>
+        <v>289</v>
       </c>
     </row>
     <row r="25" spans="1:11">
@@ -2437,10 +2461,10 @@
         <v>56</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E25" s="1" t="s">
-        <v>158</v>
+        <v>161</v>
       </c>
       <c r="F25" s="1">
         <v>0</v>
@@ -2452,10 +2476,10 @@
         <v>113</v>
       </c>
       <c r="I25" s="1" t="s">
-        <v>247</v>
+        <v>253</v>
       </c>
       <c r="J25" s="1" t="s">
-        <v>284</v>
+        <v>290</v>
       </c>
     </row>
     <row r="26" spans="1:11">
@@ -2466,10 +2490,10 @@
         <v>57</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>159</v>
+        <v>162</v>
       </c>
       <c r="F26" s="1">
         <v>0</v>
@@ -2481,10 +2505,10 @@
         <v>341</v>
       </c>
       <c r="I26" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="J26" s="1" t="s">
-        <v>285</v>
+        <v>291</v>
       </c>
     </row>
     <row r="27" spans="1:11">
@@ -2495,10 +2519,10 @@
         <v>58</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E27" s="1" t="s">
-        <v>160</v>
+        <v>163</v>
       </c>
       <c r="F27" s="1">
         <v>0</v>
@@ -2510,10 +2534,10 @@
         <v>438</v>
       </c>
       <c r="I27" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="J27" s="1" t="s">
-        <v>286</v>
+        <v>292</v>
       </c>
     </row>
     <row r="28" spans="1:11">
@@ -2524,10 +2548,10 @@
         <v>59</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E28" s="1" t="s">
-        <v>161</v>
+        <v>164</v>
       </c>
       <c r="F28" s="1">
         <v>0</v>
@@ -2539,10 +2563,10 @@
         <v>5</v>
       </c>
       <c r="I28" s="1" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="J28" s="1" t="s">
-        <v>287</v>
+        <v>293</v>
       </c>
     </row>
     <row r="29" spans="1:11">
@@ -2553,22 +2577,22 @@
         <v>60</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>162</v>
+        <v>165</v>
       </c>
       <c r="F29" s="1">
-        <v>311249</v>
+        <v>282775</v>
       </c>
       <c r="G29" s="1">
-        <v>80.7</v>
+        <v>73.3</v>
       </c>
       <c r="H29" s="1">
         <v>7</v>
       </c>
       <c r="K29" s="1" t="s">
-        <v>310</v>
+        <v>316</v>
       </c>
     </row>
     <row r="30" spans="1:11">
@@ -2579,10 +2603,10 @@
         <v>61</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>163</v>
+        <v>166</v>
       </c>
       <c r="F30" s="1">
         <v>0</v>
@@ -2594,7 +2618,7 @@
         <v>3</v>
       </c>
       <c r="K30" s="1" t="s">
-        <v>311</v>
+        <v>317</v>
       </c>
     </row>
     <row r="31" spans="1:11">
@@ -2605,10 +2629,10 @@
         <v>62</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E31" s="1" t="s">
-        <v>164</v>
+        <v>167</v>
       </c>
       <c r="F31" s="1">
         <v>0</v>
@@ -2620,7 +2644,7 @@
         <v>2</v>
       </c>
       <c r="K31" s="1" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
     </row>
     <row r="32" spans="1:11">
@@ -2631,10 +2655,10 @@
         <v>63</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E32" s="1" t="s">
-        <v>165</v>
+        <v>168</v>
       </c>
       <c r="F32" s="1">
         <v>0</v>
@@ -2646,7 +2670,7 @@
         <v>2</v>
       </c>
       <c r="K32" s="1" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
     </row>
     <row r="33" spans="1:11">
@@ -2657,10 +2681,10 @@
         <v>64</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E33" s="1" t="s">
-        <v>166</v>
+        <v>169</v>
       </c>
       <c r="F33" s="1">
         <v>0</v>
@@ -2672,7 +2696,7 @@
         <v>2</v>
       </c>
       <c r="K33" s="1" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
     </row>
     <row r="34" spans="1:11">
@@ -2683,13 +2707,13 @@
         <v>11</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>131</v>
+        <v>134</v>
       </c>
       <c r="E34" s="1" t="s">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="F34" s="1">
         <v>0</v>
@@ -2701,10 +2725,10 @@
         <v>385595</v>
       </c>
       <c r="I34" s="1" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="J34" s="1" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
     </row>
     <row r="35" spans="1:11">
@@ -2715,13 +2739,13 @@
         <v>65</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E35" s="1" t="s">
-        <v>168</v>
+        <v>171</v>
       </c>
       <c r="F35" s="1">
         <v>0</v>
@@ -2733,10 +2757,10 @@
         <v>4</v>
       </c>
       <c r="I35" s="1" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="J35" s="1" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
     </row>
     <row r="36" spans="1:11">
@@ -2747,13 +2771,13 @@
         <v>14</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>132</v>
+        <v>135</v>
       </c>
       <c r="E36" s="1" t="s">
-        <v>169</v>
+        <v>172</v>
       </c>
       <c r="F36" s="1">
         <v>0</v>
@@ -2765,10 +2789,10 @@
         <v>30</v>
       </c>
       <c r="I36" s="1" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="J36" s="1" t="s">
-        <v>288</v>
+        <v>294</v>
       </c>
     </row>
     <row r="37" spans="1:11">
@@ -2779,10 +2803,10 @@
         <v>66</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E37" s="1" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="F37" s="1">
         <v>0</v>
@@ -2794,10 +2818,10 @@
         <v>1</v>
       </c>
       <c r="I37" s="1" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
       <c r="J37" s="1" t="s">
-        <v>234</v>
+        <v>240</v>
       </c>
     </row>
     <row r="38" spans="1:11">
@@ -2808,10 +2832,10 @@
         <v>67</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="F38" s="1">
         <v>0</v>
@@ -2823,10 +2847,10 @@
         <v>95</v>
       </c>
       <c r="I38" s="1" t="s">
-        <v>248</v>
+        <v>254</v>
       </c>
       <c r="J38" s="1" t="s">
-        <v>289</v>
+        <v>295</v>
       </c>
     </row>
     <row r="39" spans="1:11">
@@ -2837,10 +2861,10 @@
         <v>68</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="F39" s="1">
         <v>0</v>
@@ -2849,13 +2873,13 @@
         <v>0</v>
       </c>
       <c r="H39" s="1">
-        <v>1794</v>
+        <v>1790</v>
       </c>
       <c r="I39" s="1" t="s">
-        <v>241</v>
+        <v>247</v>
       </c>
       <c r="J39" s="1" t="s">
-        <v>290</v>
+        <v>296</v>
       </c>
     </row>
     <row r="40" spans="1:11">
@@ -2866,10 +2890,10 @@
         <v>69</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="F40" s="1">
         <v>0</v>
@@ -2878,13 +2902,13 @@
         <v>0</v>
       </c>
       <c r="H40" s="1">
-        <v>8112</v>
+        <v>6967</v>
       </c>
       <c r="I40" s="1" t="s">
-        <v>242</v>
+        <v>248</v>
       </c>
       <c r="J40" s="1" t="s">
-        <v>291</v>
+        <v>297</v>
       </c>
     </row>
     <row r="41" spans="1:11">
@@ -2895,10 +2919,10 @@
         <v>70</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="F41" s="1">
         <v>0</v>
@@ -2910,10 +2934,10 @@
         <v>5</v>
       </c>
       <c r="I41" s="1" t="s">
-        <v>238</v>
+        <v>244</v>
       </c>
       <c r="J41" s="1" t="s">
-        <v>251</v>
+        <v>258</v>
       </c>
     </row>
     <row r="42" spans="1:11">
@@ -2924,10 +2948,10 @@
         <v>71</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F42" s="1">
         <v>0</v>
@@ -2939,7 +2963,7 @@
         <v>4</v>
       </c>
       <c r="K42" s="1" t="s">
-        <v>313</v>
+        <v>319</v>
       </c>
     </row>
     <row r="43" spans="1:11">
@@ -2950,10 +2974,10 @@
         <v>72</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
       <c r="F43" s="1">
         <v>0</v>
@@ -2965,7 +2989,7 @@
         <v>3</v>
       </c>
       <c r="K43" s="1" t="s">
-        <v>314</v>
+        <v>320</v>
       </c>
     </row>
     <row r="44" spans="1:11">
@@ -2976,10 +3000,10 @@
         <v>73</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="F44" s="1">
         <v>0</v>
@@ -2988,13 +3012,13 @@
         <v>0</v>
       </c>
       <c r="H44" s="1">
-        <v>3829</v>
+        <v>3275</v>
       </c>
       <c r="I44" s="1" t="s">
-        <v>243</v>
+        <v>249</v>
       </c>
       <c r="J44" s="1" t="s">
-        <v>292</v>
+        <v>298</v>
       </c>
     </row>
     <row r="45" spans="1:11">
@@ -3005,10 +3029,10 @@
         <v>36</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>124</v>
+        <v>127</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="F45" s="1">
         <v>0</v>
@@ -3020,10 +3044,10 @@
         <v>380766</v>
       </c>
       <c r="I45" s="1" t="s">
-        <v>235</v>
+        <v>241</v>
       </c>
       <c r="J45" s="1" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
     </row>
     <row r="46" spans="1:11">
@@ -3034,13 +3058,13 @@
         <v>13</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E46" s="1" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="F46" s="1">
         <v>0</v>
@@ -3052,10 +3076,10 @@
         <v>6000</v>
       </c>
       <c r="I46" s="1" t="s">
-        <v>249</v>
+        <v>245</v>
       </c>
       <c r="J46" s="1" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
     </row>
     <row r="47" spans="1:11">
@@ -3066,10 +3090,10 @@
         <v>74</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="F47" s="1">
         <v>0</v>
@@ -3081,7 +3105,7 @@
         <v>4</v>
       </c>
       <c r="K47" s="1" t="s">
-        <v>315</v>
+        <v>321</v>
       </c>
     </row>
     <row r="48" spans="1:11">
@@ -3092,10 +3116,10 @@
         <v>75</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="F48" s="1">
         <v>0</v>
@@ -3104,10 +3128,13 @@
         <v>0</v>
       </c>
       <c r="H48" s="1">
-        <v>2</v>
-      </c>
-      <c r="K48" s="1" t="s">
-        <v>316</v>
+        <v>4275</v>
+      </c>
+      <c r="I48" s="1" t="s">
+        <v>255</v>
+      </c>
+      <c r="J48" s="1" t="s">
+        <v>299</v>
       </c>
     </row>
     <row r="49" spans="1:11">
@@ -3118,10 +3145,10 @@
         <v>76</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E49" s="1" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="F49" s="1">
         <v>0</v>
@@ -3130,10 +3157,10 @@
         <v>0</v>
       </c>
       <c r="H49" s="1">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K49" s="1" t="s">
-        <v>317</v>
+        <v>322</v>
       </c>
     </row>
     <row r="50" spans="1:11">
@@ -3144,10 +3171,10 @@
         <v>77</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E50" s="1" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="F50" s="1">
         <v>0</v>
@@ -3156,10 +3183,10 @@
         <v>0</v>
       </c>
       <c r="H50" s="1">
-        <v>4</v>
+        <v>6000</v>
       </c>
       <c r="K50" s="1" t="s">
-        <v>318</v>
+        <v>323</v>
       </c>
     </row>
     <row r="51" spans="1:11">
@@ -3170,10 +3197,10 @@
         <v>78</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E51" s="1" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="F51" s="1">
         <v>0</v>
@@ -3182,10 +3209,10 @@
         <v>0</v>
       </c>
       <c r="H51" s="1">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="K51" s="1" t="s">
-        <v>319</v>
+        <v>324</v>
       </c>
     </row>
     <row r="52" spans="1:11">
@@ -3196,10 +3223,10 @@
         <v>79</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E52" s="1" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="F52" s="1">
         <v>0</v>
@@ -3208,10 +3235,10 @@
         <v>0</v>
       </c>
       <c r="H52" s="1">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="K52" s="1" t="s">
-        <v>312</v>
+        <v>325</v>
       </c>
     </row>
     <row r="53" spans="1:11">
@@ -3222,10 +3249,10 @@
         <v>80</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="E53" s="1" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="F53" s="1">
         <v>0</v>
@@ -3234,10 +3261,10 @@
         <v>0</v>
       </c>
       <c r="H53" s="1">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="K53" s="1" t="s">
-        <v>320</v>
+        <v>326</v>
       </c>
     </row>
     <row r="54" spans="1:11">
@@ -3248,10 +3275,10 @@
         <v>81</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E54" s="1" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="F54" s="1">
         <v>0</v>
@@ -3260,30 +3287,24 @@
         <v>0</v>
       </c>
       <c r="H54" s="1">
-        <v>364</v>
-      </c>
-      <c r="I54" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="J54" s="1" t="s">
-        <v>293</v>
+        <v>2</v>
+      </c>
+      <c r="K54" s="1" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="55" spans="1:11">
       <c r="A55" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>14</v>
+        <v>82</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D55" s="1" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E55" s="1" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="F55" s="1">
         <v>0</v>
@@ -3292,27 +3313,24 @@
         <v>0</v>
       </c>
       <c r="H55" s="1">
-        <v>30</v>
-      </c>
-      <c r="I55" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="J55" s="1" t="s">
-        <v>288</v>
+        <v>3</v>
+      </c>
+      <c r="K55" s="1" t="s">
+        <v>327</v>
       </c>
     </row>
     <row r="56" spans="1:11">
       <c r="A56" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E56" s="1" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="F56" s="1">
         <v>0</v>
@@ -3321,24 +3339,30 @@
         <v>0</v>
       </c>
       <c r="H56" s="1">
-        <v>30</v>
-      </c>
-      <c r="K56" s="1" t="s">
-        <v>321</v>
+        <v>656</v>
+      </c>
+      <c r="I56" s="1" t="s">
+        <v>256</v>
+      </c>
+      <c r="J56" s="1" t="s">
+        <v>275</v>
       </c>
     </row>
     <row r="57" spans="1:11">
       <c r="A57" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C57" s="1" t="s">
         <v>126</v>
       </c>
+      <c r="D57" s="1" t="s">
+        <v>132</v>
+      </c>
       <c r="E57" s="1" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="F57" s="1">
         <v>0</v>
@@ -3347,10 +3371,13 @@
         <v>0</v>
       </c>
       <c r="H57" s="1">
-        <v>5</v>
-      </c>
-      <c r="K57" s="1" t="s">
-        <v>322</v>
+        <v>6</v>
+      </c>
+      <c r="I57" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="J57" s="1" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="58" spans="1:11">
@@ -3358,13 +3385,16 @@
         <v>7</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>84</v>
+        <v>14</v>
       </c>
       <c r="C58" s="1" t="s">
         <v>126</v>
       </c>
+      <c r="D58" s="1" t="s">
+        <v>131</v>
+      </c>
       <c r="E58" s="1" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="F58" s="1">
         <v>0</v>
@@ -3373,10 +3403,13 @@
         <v>0</v>
       </c>
       <c r="H58" s="1">
-        <v>15</v>
-      </c>
-      <c r="K58" s="1" t="s">
-        <v>323</v>
+        <v>30</v>
+      </c>
+      <c r="I58" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="J58" s="1" t="s">
+        <v>294</v>
       </c>
     </row>
     <row r="59" spans="1:11">
@@ -3387,10 +3420,10 @@
         <v>85</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="F59" s="1">
         <v>0</v>
@@ -3399,10 +3432,10 @@
         <v>0</v>
       </c>
       <c r="H59" s="1">
-        <v>2</v>
+        <v>30</v>
       </c>
       <c r="K59" s="1" t="s">
-        <v>312</v>
+        <v>328</v>
       </c>
     </row>
     <row r="60" spans="1:11">
@@ -3413,10 +3446,10 @@
         <v>86</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E60" s="1" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="F60" s="1">
         <v>0</v>
@@ -3425,10 +3458,10 @@
         <v>0</v>
       </c>
       <c r="H60" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K60" s="1" t="s">
-        <v>312</v>
+        <v>329</v>
       </c>
     </row>
     <row r="61" spans="1:11">
@@ -3439,10 +3472,10 @@
         <v>87</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E61" s="1" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="F61" s="1">
         <v>0</v>
@@ -3451,10 +3484,10 @@
         <v>0</v>
       </c>
       <c r="H61" s="1">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="K61" s="1" t="s">
-        <v>312</v>
+        <v>330</v>
       </c>
     </row>
     <row r="62" spans="1:11">
@@ -3465,10 +3498,10 @@
         <v>88</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="F62" s="1">
         <v>0</v>
@@ -3480,7 +3513,7 @@
         <v>2</v>
       </c>
       <c r="K62" s="1" t="s">
-        <v>312</v>
+        <v>318</v>
       </c>
     </row>
     <row r="63" spans="1:11">
@@ -3494,7 +3527,7 @@
         <v>126</v>
       </c>
       <c r="E63" s="1" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="F63" s="1">
         <v>0</v>
@@ -3506,7 +3539,7 @@
         <v>2</v>
       </c>
       <c r="K63" s="1" t="s">
-        <v>324</v>
+        <v>318</v>
       </c>
     </row>
     <row r="64" spans="1:11">
@@ -3517,10 +3550,10 @@
         <v>90</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E64" s="1" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="F64" s="1">
         <v>0</v>
@@ -3531,11 +3564,8 @@
       <c r="H64" s="1">
         <v>2</v>
       </c>
-      <c r="I64" s="1" t="s">
-        <v>250</v>
-      </c>
-      <c r="J64" s="1" t="s">
-        <v>294</v>
+      <c r="K64" s="1" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="65" spans="1:11">
@@ -3546,10 +3576,10 @@
         <v>91</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E65" s="1" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="F65" s="1">
         <v>0</v>
@@ -3558,13 +3588,10 @@
         <v>0</v>
       </c>
       <c r="H65" s="1">
-        <v>12</v>
-      </c>
-      <c r="I65" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="J65" s="1" t="s">
-        <v>295</v>
+        <v>2</v>
+      </c>
+      <c r="K65" s="1" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="66" spans="1:11">
@@ -3575,10 +3602,10 @@
         <v>92</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E66" s="1" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="F66" s="1">
         <v>0</v>
@@ -3587,13 +3614,10 @@
         <v>0</v>
       </c>
       <c r="H66" s="1">
-        <v>1</v>
-      </c>
-      <c r="I66" s="1" t="s">
-        <v>238</v>
-      </c>
-      <c r="J66" s="1" t="s">
-        <v>238</v>
+        <v>2</v>
+      </c>
+      <c r="K66" s="1" t="s">
+        <v>331</v>
       </c>
     </row>
     <row r="67" spans="1:11">
@@ -3604,10 +3628,10 @@
         <v>93</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="F67" s="1">
         <v>0</v>
@@ -3616,13 +3640,13 @@
         <v>0</v>
       </c>
       <c r="H67" s="1">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="I67" s="1" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="J67" s="1" t="s">
-        <v>251</v>
+        <v>300</v>
       </c>
     </row>
     <row r="68" spans="1:11">
@@ -3636,7 +3660,7 @@
         <v>126</v>
       </c>
       <c r="E68" s="1" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="F68" s="1">
         <v>0</v>
@@ -3645,10 +3669,13 @@
         <v>0</v>
       </c>
       <c r="H68" s="1">
-        <v>3</v>
-      </c>
-      <c r="K68" s="1" t="s">
-        <v>325</v>
+        <v>12</v>
+      </c>
+      <c r="I68" s="1" t="s">
+        <v>254</v>
+      </c>
+      <c r="J68" s="1" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="69" spans="1:11">
@@ -3659,10 +3686,10 @@
         <v>95</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E69" s="1" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="F69" s="1">
         <v>0</v>
@@ -3671,10 +3698,13 @@
         <v>0</v>
       </c>
       <c r="H69" s="1">
-        <v>2</v>
-      </c>
-      <c r="K69" s="1" t="s">
-        <v>312</v>
+        <v>1</v>
+      </c>
+      <c r="I69" s="1" t="s">
+        <v>244</v>
+      </c>
+      <c r="J69" s="1" t="s">
+        <v>244</v>
       </c>
     </row>
     <row r="70" spans="1:11">
@@ -3685,10 +3715,10 @@
         <v>96</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="F70" s="1">
         <v>0</v>
@@ -3697,10 +3727,13 @@
         <v>0</v>
       </c>
       <c r="H70" s="1">
-        <v>2</v>
-      </c>
-      <c r="K70" s="1" t="s">
-        <v>312</v>
+        <v>1</v>
+      </c>
+      <c r="I70" s="1" t="s">
+        <v>258</v>
+      </c>
+      <c r="J70" s="1" t="s">
+        <v>258</v>
       </c>
     </row>
     <row r="71" spans="1:11">
@@ -3711,10 +3744,10 @@
         <v>97</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="F71" s="1">
         <v>0</v>
@@ -3723,10 +3756,10 @@
         <v>0</v>
       </c>
       <c r="H71" s="1">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="K71" s="1" t="s">
-        <v>312</v>
+        <v>332</v>
       </c>
     </row>
     <row r="72" spans="1:11">
@@ -3737,10 +3770,10 @@
         <v>98</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="F72" s="1">
         <v>0</v>
@@ -3749,30 +3782,24 @@
         <v>0</v>
       </c>
       <c r="H72" s="1">
-        <v>7</v>
-      </c>
-      <c r="I72" s="1" t="s">
-        <v>236</v>
-      </c>
-      <c r="J72" s="1" t="s">
-        <v>296</v>
+        <v>2</v>
+      </c>
+      <c r="K72" s="1" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="73" spans="1:11">
       <c r="A73" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>15</v>
+        <v>99</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D73" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="E73" s="1" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="F73" s="1">
         <v>0</v>
@@ -3781,27 +3808,24 @@
         <v>0</v>
       </c>
       <c r="H73" s="1">
-        <v>6</v>
-      </c>
-      <c r="I73" s="1" t="s">
-        <v>234</v>
-      </c>
-      <c r="J73" s="1" t="s">
-        <v>252</v>
+        <v>2</v>
+      </c>
+      <c r="K73" s="1" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="74" spans="1:11">
       <c r="A74" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="C74" s="1" t="s">
         <v>126</v>
       </c>
       <c r="E74" s="1" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="F74" s="1">
         <v>0</v>
@@ -3810,24 +3834,24 @@
         <v>0</v>
       </c>
       <c r="H74" s="1">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="K74" s="1" t="s">
-        <v>326</v>
+        <v>318</v>
       </c>
     </row>
     <row r="75" spans="1:11">
       <c r="A75" s="1" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="F75" s="1">
         <v>0</v>
@@ -3836,10 +3860,13 @@
         <v>0</v>
       </c>
       <c r="H75" s="1">
-        <v>5</v>
-      </c>
-      <c r="K75" s="1" t="s">
-        <v>327</v>
+        <v>7</v>
+      </c>
+      <c r="I75" s="1" t="s">
+        <v>242</v>
+      </c>
+      <c r="J75" s="1" t="s">
+        <v>302</v>
       </c>
     </row>
     <row r="76" spans="1:11">
@@ -3847,13 +3874,16 @@
         <v>8</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>101</v>
+        <v>15</v>
       </c>
       <c r="C76" s="1" t="s">
         <v>126</v>
       </c>
+      <c r="D76" s="1" t="s">
+        <v>131</v>
+      </c>
       <c r="E76" s="1" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="F76" s="1">
         <v>0</v>
@@ -3862,10 +3892,13 @@
         <v>0</v>
       </c>
       <c r="H76" s="1">
-        <v>5</v>
-      </c>
-      <c r="K76" s="1" t="s">
-        <v>328</v>
+        <v>6</v>
+      </c>
+      <c r="I76" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="J76" s="1" t="s">
+        <v>259</v>
       </c>
     </row>
     <row r="77" spans="1:11">
@@ -3876,10 +3909,10 @@
         <v>102</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E77" s="1" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="F77" s="1">
         <v>0</v>
@@ -3890,11 +3923,8 @@
       <c r="H77" s="1">
         <v>6</v>
       </c>
-      <c r="I77" s="1" t="s">
-        <v>252</v>
-      </c>
-      <c r="J77" s="1" t="s">
-        <v>297</v>
+      <c r="K77" s="1" t="s">
+        <v>333</v>
       </c>
     </row>
     <row r="78" spans="1:11">
@@ -3905,10 +3935,10 @@
         <v>103</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>123</v>
+        <v>129</v>
       </c>
       <c r="E78" s="1" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="F78" s="1">
         <v>0</v>
@@ -3917,10 +3947,10 @@
         <v>0</v>
       </c>
       <c r="H78" s="1">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="K78" s="1" t="s">
-        <v>312</v>
+        <v>334</v>
       </c>
     </row>
     <row r="79" spans="1:11">
@@ -3931,10 +3961,10 @@
         <v>104</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="E79" s="1" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="F79" s="1">
         <v>0</v>
@@ -3945,11 +3975,8 @@
       <c r="H79" s="1">
         <v>5</v>
       </c>
-      <c r="I79" s="1" t="s">
-        <v>253</v>
-      </c>
-      <c r="J79" s="1" t="s">
-        <v>298</v>
+      <c r="K79" s="1" t="s">
+        <v>335</v>
       </c>
     </row>
     <row r="80" spans="1:11">
@@ -3960,10 +3987,10 @@
         <v>105</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E80" s="1" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="F80" s="1">
         <v>0</v>
@@ -3975,10 +4002,10 @@
         <v>6</v>
       </c>
       <c r="I80" s="1" t="s">
-        <v>254</v>
+        <v>259</v>
       </c>
       <c r="J80" s="1" t="s">
-        <v>299</v>
+        <v>303</v>
       </c>
     </row>
     <row r="81" spans="1:11">
@@ -3989,10 +4016,10 @@
         <v>106</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E81" s="1" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="F81" s="1">
         <v>0</v>
@@ -4001,13 +4028,10 @@
         <v>0</v>
       </c>
       <c r="H81" s="1">
-        <v>5</v>
-      </c>
-      <c r="I81" s="1" t="s">
-        <v>255</v>
-      </c>
-      <c r="J81" s="1" t="s">
-        <v>298</v>
+        <v>2</v>
+      </c>
+      <c r="K81" s="1" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="82" spans="1:11">
@@ -4018,10 +4042,10 @@
         <v>107</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>125</v>
+        <v>130</v>
       </c>
       <c r="E82" s="1" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="F82" s="1">
         <v>0</v>
@@ -4030,13 +4054,13 @@
         <v>0</v>
       </c>
       <c r="H82" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I82" s="1" t="s">
-        <v>256</v>
+        <v>260</v>
       </c>
       <c r="J82" s="1" t="s">
-        <v>300</v>
+        <v>304</v>
       </c>
     </row>
     <row r="83" spans="1:11">
@@ -4047,10 +4071,10 @@
         <v>108</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="E83" s="1" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="F83" s="1">
         <v>0</v>
@@ -4059,10 +4083,13 @@
         <v>0</v>
       </c>
       <c r="H83" s="1">
-        <v>2</v>
-      </c>
-      <c r="K83" s="1" t="s">
-        <v>312</v>
+        <v>6</v>
+      </c>
+      <c r="I83" s="1" t="s">
+        <v>261</v>
+      </c>
+      <c r="J83" s="1" t="s">
+        <v>305</v>
       </c>
     </row>
     <row r="84" spans="1:11">
@@ -4073,10 +4100,10 @@
         <v>109</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>123</v>
+        <v>130</v>
       </c>
       <c r="E84" s="1" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="F84" s="1">
         <v>0</v>
@@ -4085,13 +4112,13 @@
         <v>0</v>
       </c>
       <c r="H84" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I84" s="1" t="s">
-        <v>257</v>
+        <v>262</v>
       </c>
       <c r="J84" s="1" t="s">
-        <v>251</v>
+        <v>304</v>
       </c>
     </row>
     <row r="85" spans="1:11">
@@ -4102,10 +4129,10 @@
         <v>110</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>123</v>
+        <v>128</v>
       </c>
       <c r="E85" s="1" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="F85" s="1">
         <v>0</v>
@@ -4117,10 +4144,10 @@
         <v>6</v>
       </c>
       <c r="I85" s="1" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="J85" s="1" t="s">
-        <v>301</v>
+        <v>306</v>
       </c>
     </row>
     <row r="86" spans="1:11">
@@ -4131,10 +4158,10 @@
         <v>111</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E86" s="1" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="F86" s="1">
         <v>0</v>
@@ -4143,13 +4170,10 @@
         <v>0</v>
       </c>
       <c r="H86" s="1">
-        <v>5</v>
-      </c>
-      <c r="I86" s="1" t="s">
-        <v>259</v>
-      </c>
-      <c r="J86" s="1" t="s">
-        <v>271</v>
+        <v>2</v>
+      </c>
+      <c r="K86" s="1" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="87" spans="1:11">
@@ -4160,10 +4184,10 @@
         <v>112</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E87" s="1" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="F87" s="1">
         <v>0</v>
@@ -4172,13 +4196,13 @@
         <v>0</v>
       </c>
       <c r="H87" s="1">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="I87" s="1" t="s">
-        <v>260</v>
+        <v>263</v>
       </c>
       <c r="J87" s="1" t="s">
-        <v>302</v>
+        <v>258</v>
       </c>
     </row>
     <row r="88" spans="1:11">
@@ -4189,10 +4213,10 @@
         <v>113</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E88" s="1" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="F88" s="1">
         <v>0</v>
@@ -4204,10 +4228,10 @@
         <v>6</v>
       </c>
       <c r="I88" s="1" t="s">
-        <v>261</v>
+        <v>264</v>
       </c>
       <c r="J88" s="1" t="s">
-        <v>303</v>
+        <v>307</v>
       </c>
     </row>
     <row r="89" spans="1:11">
@@ -4218,10 +4242,10 @@
         <v>114</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E89" s="1" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="F89" s="1">
         <v>0</v>
@@ -4230,13 +4254,13 @@
         <v>0</v>
       </c>
       <c r="H89" s="1">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="I89" s="1" t="s">
-        <v>262</v>
+        <v>265</v>
       </c>
       <c r="J89" s="1" t="s">
-        <v>250</v>
+        <v>277</v>
       </c>
     </row>
     <row r="90" spans="1:11">
@@ -4247,10 +4271,10 @@
         <v>115</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E90" s="1" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="F90" s="1">
         <v>0</v>
@@ -4259,13 +4283,13 @@
         <v>0</v>
       </c>
       <c r="H90" s="1">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="I90" s="1" t="s">
-        <v>234</v>
+        <v>266</v>
       </c>
       <c r="J90" s="1" t="s">
-        <v>259</v>
+        <v>308</v>
       </c>
     </row>
     <row r="91" spans="1:11">
@@ -4276,10 +4300,10 @@
         <v>116</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="E91" s="1" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="F91" s="1">
         <v>0</v>
@@ -4291,10 +4315,10 @@
         <v>6</v>
       </c>
       <c r="I91" s="1" t="s">
-        <v>263</v>
+        <v>267</v>
       </c>
       <c r="J91" s="1" t="s">
-        <v>245</v>
+        <v>309</v>
       </c>
     </row>
     <row r="92" spans="1:11">
@@ -4305,10 +4329,10 @@
         <v>117</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E92" s="1" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="F92" s="1">
         <v>0</v>
@@ -4317,10 +4341,13 @@
         <v>0</v>
       </c>
       <c r="H92" s="1">
-        <v>2</v>
-      </c>
-      <c r="K92" s="1" t="s">
-        <v>312</v>
+        <v>6</v>
+      </c>
+      <c r="I92" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="J92" s="1" t="s">
+        <v>257</v>
       </c>
     </row>
     <row r="93" spans="1:11">
@@ -4331,10 +4358,10 @@
         <v>118</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E93" s="1" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="F93" s="1">
         <v>0</v>
@@ -4343,30 +4370,27 @@
         <v>0</v>
       </c>
       <c r="H93" s="1">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="I93" s="1" t="s">
-        <v>264</v>
+        <v>240</v>
       </c>
       <c r="J93" s="1" t="s">
-        <v>304</v>
+        <v>265</v>
       </c>
     </row>
     <row r="94" spans="1:11">
       <c r="A94" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>14</v>
+        <v>119</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D94" s="1" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E94" s="1" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="F94" s="1">
         <v>0</v>
@@ -4375,27 +4399,27 @@
         <v>0</v>
       </c>
       <c r="H94" s="1">
-        <v>30</v>
+        <v>6</v>
       </c>
       <c r="I94" s="1" t="s">
-        <v>234</v>
+        <v>269</v>
       </c>
       <c r="J94" s="1" t="s">
-        <v>288</v>
+        <v>251</v>
       </c>
     </row>
     <row r="95" spans="1:11">
       <c r="A95" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>91</v>
+        <v>120</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>123</v>
+        <v>126</v>
       </c>
       <c r="E95" s="1" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="F95" s="1">
         <v>0</v>
@@ -4404,30 +4428,24 @@
         <v>0</v>
       </c>
       <c r="H95" s="1">
-        <v>14</v>
-      </c>
-      <c r="I95" s="1" t="s">
-        <v>248</v>
-      </c>
-      <c r="J95" s="1" t="s">
-        <v>305</v>
+        <v>2</v>
+      </c>
+      <c r="K95" s="1" t="s">
+        <v>318</v>
       </c>
     </row>
     <row r="96" spans="1:11">
       <c r="A96" s="1" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="D96" s="1" t="s">
         <v>128</v>
       </c>
       <c r="E96" s="1" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="F96" s="1">
         <v>0</v>
@@ -4436,13 +4454,13 @@
         <v>0</v>
       </c>
       <c r="H96" s="1">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="I96" s="1" t="s">
-        <v>236</v>
+        <v>270</v>
       </c>
       <c r="J96" s="1" t="s">
-        <v>296</v>
+        <v>310</v>
       </c>
     </row>
     <row r="97" spans="1:11">
@@ -4450,45 +4468,45 @@
         <v>9</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>120</v>
+        <v>14</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>125</v>
+        <v>126</v>
+      </c>
+      <c r="D97" s="1" t="s">
+        <v>136</v>
       </c>
       <c r="E97" s="1" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="F97" s="1">
+        <v>0</v>
+      </c>
+      <c r="G97" s="1">
+        <v>0</v>
+      </c>
+      <c r="H97" s="1">
         <v>30</v>
       </c>
-      <c r="G97" s="1">
-        <v>60</v>
-      </c>
-      <c r="H97" s="1">
-        <v>1</v>
-      </c>
       <c r="I97" s="1" t="s">
-        <v>265</v>
+        <v>240</v>
       </c>
       <c r="J97" s="1" t="s">
-        <v>265</v>
+        <v>294</v>
       </c>
     </row>
     <row r="98" spans="1:11">
       <c r="A98" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>15</v>
+        <v>94</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>123</v>
-      </c>
-      <c r="D98" s="1" t="s">
-        <v>134</v>
+        <v>126</v>
       </c>
       <c r="E98" s="1" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="F98" s="1">
         <v>0</v>
@@ -4497,30 +4515,30 @@
         <v>0</v>
       </c>
       <c r="H98" s="1">
-        <v>6</v>
+        <v>14</v>
       </c>
       <c r="I98" s="1" t="s">
-        <v>234</v>
+        <v>254</v>
       </c>
       <c r="J98" s="1" t="s">
-        <v>252</v>
+        <v>311</v>
       </c>
     </row>
     <row r="99" spans="1:11">
       <c r="A99" s="1" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>125</v>
+        <v>128</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="F99" s="1">
         <v>0</v>
@@ -4529,50 +4547,143 @@
         <v>0</v>
       </c>
       <c r="H99" s="1">
-        <v>14</v>
+        <v>8</v>
       </c>
       <c r="I99" s="1" t="s">
-        <v>266</v>
+        <v>242</v>
       </c>
       <c r="J99" s="1" t="s">
-        <v>306</v>
+        <v>302</v>
       </c>
     </row>
     <row r="100" spans="1:11">
       <c r="A100" s="1" t="s">
+        <v>9</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>123</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="E100" s="1" t="s">
+        <v>236</v>
+      </c>
+      <c r="F100" s="1">
+        <v>30</v>
+      </c>
+      <c r="G100" s="1">
+        <v>60</v>
+      </c>
+      <c r="H100" s="1">
+        <v>1</v>
+      </c>
+      <c r="I100" s="1" t="s">
+        <v>271</v>
+      </c>
+      <c r="J100" s="1" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="101" spans="1:11">
+      <c r="A101" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="B100" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C100" s="1" t="s">
+      <c r="B101" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C101" s="1" t="s">
         <v>126</v>
       </c>
-      <c r="E100" s="1" t="s">
-        <v>233</v>
-      </c>
-      <c r="F100" s="1">
-        <v>0</v>
-      </c>
-      <c r="G100" s="1">
-        <v>0</v>
-      </c>
-      <c r="H100" s="1">
+      <c r="D101" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="E101" s="1" t="s">
+        <v>237</v>
+      </c>
+      <c r="F101" s="1">
+        <v>0</v>
+      </c>
+      <c r="G101" s="1">
+        <v>0</v>
+      </c>
+      <c r="H101" s="1">
+        <v>6</v>
+      </c>
+      <c r="I101" s="1" t="s">
+        <v>240</v>
+      </c>
+      <c r="J101" s="1" t="s">
+        <v>259</v>
+      </c>
+    </row>
+    <row r="102" spans="1:11">
+      <c r="A102" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B102" s="1" t="s">
+        <v>124</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="D102" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="E102" s="1" t="s">
+        <v>238</v>
+      </c>
+      <c r="F102" s="1">
+        <v>0</v>
+      </c>
+      <c r="G102" s="1">
+        <v>0</v>
+      </c>
+      <c r="H102" s="1">
+        <v>14</v>
+      </c>
+      <c r="I102" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="J102" s="1" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="103" spans="1:11">
+      <c r="A103" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="B103" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>129</v>
+      </c>
+      <c r="E103" s="1" t="s">
+        <v>239</v>
+      </c>
+      <c r="F103" s="1">
+        <v>0</v>
+      </c>
+      <c r="G103" s="1">
+        <v>0</v>
+      </c>
+      <c r="H103" s="1">
         <v>5</v>
       </c>
-      <c r="K100" s="1" t="s">
-        <v>329</v>
+      <c r="K103" s="1" t="s">
+        <v>336</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K100"/>
+  <autoFilter ref="A1:K103"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:E7"/>
+  <dimension ref="A1:E8"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="30.7109375" style="1" customWidth="1"/>
@@ -4584,30 +4695,30 @@
   <sheetData>
     <row r="1" spans="1:5">
       <c r="A1" s="3" t="s">
-        <v>330</v>
+        <v>337</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>331</v>
+        <v>338</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>332</v>
+        <v>339</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>333</v>
+        <v>340</v>
       </c>
       <c r="E1" s="3" t="s">
-        <v>334</v>
+        <v>341</v>
       </c>
     </row>
     <row r="2" spans="1:5">
       <c r="A2" s="1" t="s">
-        <v>335</v>
+        <v>342</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="E2" s="1">
         <v>0</v>
@@ -4615,16 +4726,16 @@
     </row>
     <row r="3" spans="1:5">
       <c r="A3" s="1" t="s">
-        <v>336</v>
+        <v>343</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>342</v>
+        <v>350</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>346</v>
+        <v>354</v>
       </c>
       <c r="E3" s="1">
         <v>0</v>
@@ -4632,13 +4743,13 @@
     </row>
     <row r="4" spans="1:5">
       <c r="A4" s="1" t="s">
-        <v>337</v>
+        <v>344</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>343</v>
+        <v>349</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="E4" s="1">
         <v>0</v>
@@ -4646,13 +4757,13 @@
     </row>
     <row r="5" spans="1:5">
       <c r="A5" s="1" t="s">
-        <v>338</v>
+        <v>345</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>344</v>
+        <v>351</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="E5" s="1">
         <v>0</v>
@@ -4660,13 +4771,13 @@
     </row>
     <row r="6" spans="1:5">
       <c r="A6" s="1" t="s">
-        <v>339</v>
+        <v>346</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>344</v>
+        <v>352</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="E6" s="1">
         <v>0</v>
@@ -4674,20 +4785,34 @@
     </row>
     <row r="7" spans="1:5">
       <c r="A7" s="1" t="s">
-        <v>340</v>
+        <v>347</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>341</v>
+        <v>352</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>345</v>
+        <v>353</v>
       </c>
       <c r="E7" s="1">
         <v>0</v>
       </c>
     </row>
+    <row r="8" spans="1:5">
+      <c r="A8" s="1" t="s">
+        <v>348</v>
+      </c>
+      <c r="B8" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="C8" s="1" t="s">
+        <v>353</v>
+      </c>
+      <c r="E8" s="1">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:E7"/>
+  <autoFilter ref="A1:E8"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -4708,177 +4833,177 @@
         <v>27</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>347</v>
+        <v>355</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>348</v>
+        <v>356</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>349</v>
+        <v>357</v>
       </c>
     </row>
     <row r="2" spans="1:4">
       <c r="A2" s="1" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>351</v>
+        <v>359</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>358</v>
+        <v>366</v>
       </c>
       <c r="D2" s="1">
-        <v>1840</v>
+        <v>12305</v>
       </c>
     </row>
     <row r="3" spans="1:4">
       <c r="A3" s="1" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>352</v>
+        <v>360</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>359</v>
+        <v>367</v>
       </c>
       <c r="D3" s="1">
-        <v>1395</v>
+        <v>9394</v>
       </c>
     </row>
     <row r="4" spans="1:4">
       <c r="A4" s="1" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>353</v>
+        <v>361</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>360</v>
+        <v>368</v>
       </c>
       <c r="D4" s="1">
-        <v>15967</v>
+        <v>26970</v>
       </c>
     </row>
     <row r="5" spans="1:4">
       <c r="A5" s="1" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>354</v>
+        <v>362</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>361</v>
+        <v>369</v>
       </c>
       <c r="D5" s="1">
-        <v>16436</v>
+        <v>12943</v>
       </c>
     </row>
     <row r="6" spans="1:4">
       <c r="A6" s="1" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>355</v>
+        <v>363</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>362</v>
+        <v>370</v>
       </c>
       <c r="D6" s="1">
-        <v>3300</v>
+        <v>8533</v>
       </c>
     </row>
     <row r="7" spans="1:4">
       <c r="A7" s="1" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>356</v>
+        <v>364</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>363</v>
+        <v>371</v>
       </c>
       <c r="D7" s="1">
-        <v>9120</v>
+        <v>7727</v>
       </c>
     </row>
     <row r="8" spans="1:4">
       <c r="A8" s="1" t="s">
-        <v>350</v>
+        <v>358</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>357</v>
+        <v>365</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>364</v>
+        <v>372</v>
       </c>
       <c r="D8" s="1">
-        <v>26288</v>
+        <v>24948</v>
       </c>
     </row>
     <row r="9" spans="1:4">
       <c r="A9" s="1" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="B9" s="1">
         <v>1</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>365</v>
+        <v>373</v>
       </c>
     </row>
     <row r="10" spans="1:4">
       <c r="A10" s="1" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="B10" s="1">
         <v>2</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>366</v>
+        <v>374</v>
       </c>
     </row>
     <row r="11" spans="1:4">
       <c r="A11" s="1" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="B11" s="1">
         <v>3</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>367</v>
+        <v>375</v>
       </c>
     </row>
     <row r="12" spans="1:4">
       <c r="A12" s="1" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="B12" s="1">
         <v>4</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>368</v>
+        <v>376</v>
       </c>
     </row>
     <row r="13" spans="1:4">
       <c r="A13" s="1" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="B13" s="1">
         <v>5</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>369</v>
+        <v>377</v>
       </c>
     </row>
     <row r="14" spans="1:4">
       <c r="A14" s="1" t="s">
-        <v>341</v>
+        <v>349</v>
       </c>
       <c r="B14" s="1">
         <v>6</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>370</v>
+        <v>378</v>
       </c>
     </row>
   </sheetData>
@@ -4898,90 +5023,90 @@
   <sheetData>
     <row r="1" spans="1:2">
       <c r="A1" s="3" t="s">
-        <v>371</v>
+        <v>379</v>
       </c>
       <c r="B1" s="3" t="s">
-        <v>372</v>
+        <v>380</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="1" t="s">
-        <v>373</v>
+        <v>381</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>381</v>
+        <v>389</v>
       </c>
     </row>
     <row r="3" spans="1:2">
       <c r="A3" s="1" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>382</v>
+        <v>390</v>
       </c>
     </row>
     <row r="4" spans="1:2">
       <c r="A4" s="1" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>383</v>
+        <v>391</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="1" t="s">
-        <v>374</v>
+        <v>382</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>384</v>
+        <v>392</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="1" t="s">
-        <v>375</v>
+        <v>383</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>385</v>
+        <v>393</v>
       </c>
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="1" t="s">
-        <v>376</v>
+        <v>384</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>386</v>
+        <v>394</v>
       </c>
     </row>
     <row r="8" spans="1:2">
       <c r="A8" s="1" t="s">
-        <v>377</v>
+        <v>385</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>387</v>
+        <v>395</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>378</v>
+        <v>386</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>388</v>
+        <v>396</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" s="1" t="s">
-        <v>379</v>
+        <v>387</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>389</v>
+        <v>397</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" s="1" t="s">
-        <v>380</v>
+        <v>388</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>390</v>
+        <v>398</v>
       </c>
     </row>
   </sheetData>

</xml_diff>